<commit_message>
Regenerate aligned AJHB reviewer supplementary outputs
</commit_message>
<xml_diff>
--- a/production/ajhb_nwl/outputs/reviewer_revision/AJHB_reviewer_supplement_ready.xlsx
+++ b/production/ajhb_nwl/outputs/reviewer_revision/AJHB_reviewer_supplement_ready.xlsx
@@ -353,7 +353,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -364,12 +364,12 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>One measurement</t>
+          <t>One postnatal weight measurement</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Two measurements</t>
+          <t>Two postnatal weight measurements</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -403,7 +403,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Maternal age, years</t>
+          <t>Maternal age, years, mean (SD)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -430,7 +430,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Parity</t>
+          <t>Parity, mean (SD)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -457,83 +457,103 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Maternal health status: 1</t>
+          <t>Gestational age, weeks, mean (SD)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>83 (69.2%)</t>
+          <t>38.01 (3.10)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>8987 (78.3%)</t>
+          <t>39.42 (1.60)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Chi-square/Fisher</t>
+          <t>t-test</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>0.005</t>
+          <t>&lt;0.001</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Maternal health status: 2</t>
+          <t>Birthweight, g, mean (SD)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>22 (18.3%)</t>
+          <t>2880 (720)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>1820 (15.9%)</t>
+          <t>3229 (489)</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>t-test</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>&lt;0.001</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Maternal health status: 3</t>
+          <t>Preterm birth (&lt;37 weeks), n (%)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>15 (12.5%)</t>
+          <t>29 (24.0%)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>670 (5.8%)</t>
+          <t>739 (6.4%)</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Chi-square/Fisher</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>&lt;0.001</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Gestational age, weeks</t>
+          <t>Low birthweight (&lt;2500 g), n (%)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>38.01 (3.10)</t>
+          <t>29 (24.0%)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>39.42 (1.60)</t>
+          <t>707 (6.1%)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>t-test</t>
+          <t>Chi-square/Fisher</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -545,44 +565,44 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Birthweight, g</t>
+          <t>Female sex, n (%)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2880 (720)</t>
+          <t>60 (50.0%)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>3229 (489)</t>
+          <t>5886 (50.8%)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>t-test</t>
+          <t>Chi-square/Fisher</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>&lt;0.001</t>
+          <t>0.943</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Preterm birth status: term</t>
+          <t>Male sex, n (%)</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>92 (76.0%)</t>
+          <t>60 (50.0%)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>10879 (93.6%)</t>
+          <t>5712 (49.2%)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -592,41 +612,51 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>&lt;0.001</t>
+          <t>0.943</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Preterm birth status: preterm</t>
+          <t>Artificial feeding, n (%)</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>29 (24.0%)</t>
+          <t>12 (11.2%)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>739 (6.4%)</t>
+          <t>742 (6.4%)</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Chi-square/Fisher</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>&lt;0.001</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Birthweight status: normal_birthweight</t>
+          <t>Breastfeeding, n (%)</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>92 (76.0%)</t>
+          <t>80 (74.8%)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>10911 (93.9%)</t>
+          <t>9062 (78.1%)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -643,34 +673,44 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Birthweight status: low_birthweight</t>
+          <t>Mixed feeding, n (%)</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>29 (24.0%)</t>
+          <t>8 (7.5%)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>707 (6.1%)</t>
+          <t>1617 (13.9%)</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Chi-square/Fisher</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>&lt;0.001</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Neonatal sex: male</t>
+          <t>Other feeding, n (%)</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>60 (50.0%)</t>
+          <t>7 (6.5%)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>5712 (49.2%)</t>
+          <t>176 (1.5%)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -680,102 +720,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>0.943</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Neonatal sex: female</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>60 (50.0%)</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>5886 (50.8%)</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Feeding mode: breastfeeding</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>80 (74.8%)</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>9062 (78.1%)</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>Chi-square/Fisher</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>&lt;0.001</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Feeding mode: mixed</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>8 (7.5%)</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>1617 (13.9%)</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Feeding mode: artificial</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>12 (11.2%)</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>742 (6.4%)</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Feeding mode: other</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>7 (6.5%)</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>176 (1.5%)</t>
+          <t>&lt;0.001</t>
         </is>
       </c>
     </row>
@@ -824,12 +769,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Maximum neonatal weight loss, % (beta)</t>
+          <t>Linear model: maximum neonatal weight loss (%)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Pregnancy overlapping World War I: yes vs no</t>
+          <t>Pregnancy overlapped WWI</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -856,12 +801,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Maximum neonatal weight loss, % (beta)</t>
+          <t>Linear model: maximum neonatal weight loss (%)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Pregnancy overlapping influenza pandemic: yes vs no</t>
+          <t>Pregnancy overlapped influenza pandemic</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -888,12 +833,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Maximum neonatal weight loss, % (beta)</t>
+          <t>Linear model: maximum neonatal weight loss (%)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Feeding mode: breastfeeding vs artificial feeding</t>
+          <t>Breastfeeding vs artificial</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -920,12 +865,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Maximum neonatal weight loss, % (beta)</t>
+          <t>Linear model: maximum neonatal weight loss (%)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Feeding mode: mixed feeding vs artificial feeding</t>
+          <t>Mixed feeding vs artificial</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -952,12 +897,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Maximum neonatal weight loss, % (beta)</t>
+          <t>Linear model: maximum neonatal weight loss (%)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Feeding mode: other vs artificial feeding</t>
+          <t>Other feeding vs artificial</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -984,12 +929,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Maximum neonatal weight loss, % (beta)</t>
+          <t>Linear model: maximum neonatal weight loss (%)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Gestational age, weeks</t>
+          <t>Gestational age, per week</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1016,12 +961,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Maximum neonatal weight loss, % (beta)</t>
+          <t>Linear model: maximum neonatal weight loss (%)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Male sex vs female</t>
+          <t>Male vs female</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1048,7 +993,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Maximum neonatal weight loss, % (beta)</t>
+          <t>Linear model: maximum neonatal weight loss (%)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1080,12 +1025,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Maximum neonatal weight loss, % (beta)</t>
+          <t>Linear model: maximum neonatal weight loss (%)</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Maternal age, years</t>
+          <t>Maternal age, per year</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1112,12 +1057,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>High neonatal weight loss &gt;10% (odds ratio)</t>
+          <t>Logistic model: excessive neonatal weight loss &gt;10%</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Pregnancy overlapping World War I: yes vs no</t>
+          <t>Pregnancy overlapped WWI</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1144,12 +1089,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>High neonatal weight loss &gt;10% (odds ratio)</t>
+          <t>Logistic model: excessive neonatal weight loss &gt;10%</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Pregnancy overlapping influenza pandemic: yes vs no</t>
+          <t>Pregnancy overlapped influenza pandemic</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1176,12 +1121,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>High neonatal weight loss &gt;10% (odds ratio)</t>
+          <t>Logistic model: excessive neonatal weight loss &gt;10%</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Feeding mode: breastfeeding vs artificial feeding</t>
+          <t>Breastfeeding vs artificial</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1208,12 +1153,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>High neonatal weight loss &gt;10% (odds ratio)</t>
+          <t>Logistic model: excessive neonatal weight loss &gt;10%</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Feeding mode: mixed feeding vs artificial feeding</t>
+          <t>Mixed feeding vs artificial</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1240,12 +1185,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>High neonatal weight loss &gt;10% (odds ratio)</t>
+          <t>Logistic model: excessive neonatal weight loss &gt;10%</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Feeding mode: other vs artificial feeding</t>
+          <t>Other feeding vs artificial</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1272,12 +1217,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>High neonatal weight loss &gt;10% (odds ratio)</t>
+          <t>Logistic model: excessive neonatal weight loss &gt;10%</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Gestational age, weeks</t>
+          <t>Gestational age, per week</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1304,12 +1249,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>High neonatal weight loss &gt;10% (odds ratio)</t>
+          <t>Logistic model: excessive neonatal weight loss &gt;10%</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Male sex vs female</t>
+          <t>Male vs female</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1336,7 +1281,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>High neonatal weight loss &gt;10% (odds ratio)</t>
+          <t>Logistic model: excessive neonatal weight loss &gt;10%</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1368,12 +1313,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>High neonatal weight loss &gt;10% (odds ratio)</t>
+          <t>Logistic model: excessive neonatal weight loss &gt;10%</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Maternal age, years</t>
+          <t>Maternal age, per year</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">

</xml_diff>